<commit_message>
Update June data and add MPPM audit
</commit_message>
<xml_diff>
--- a/isolated_excel/LSQ Returns - Current.xlsx
+++ b/isolated_excel/LSQ Returns - Current.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Source and Method" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source and Method" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Returns'!$A$1:$E$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Returns'!$A$1:$E$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Source and Method'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2847,8 +2847,29 @@
         <v>1.0764</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>0.0639</v>
+      </c>
+      <c r="D115" s="3" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>1.0639</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E114"/>
+  <autoFilter ref="A1:E115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2898,7 +2919,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Jan 2017 to May 2026; 113 monthly observations</t>
+          <t>Jan 2017 to Jun 2026; 114 monthly observations</t>
         </is>
       </c>
     </row>

</xml_diff>